<commit_message>
MOD: Ajusta secuencia de colores
</commit_message>
<xml_diff>
--- a/outputs/programacion_franjas.xlsx
+++ b/outputs/programacion_franjas.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -505,7 +505,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_DOS_VIERNES</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -515,12 +515,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -640,16 +640,16 @@
         <v>46291</v>
       </c>
       <c r="J4" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46340</v>
+        <v>46305</v>
       </c>
       <c r="L4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M4" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -670,41 +670,41 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H5" t="n">
         <v>12</v>
       </c>
       <c r="I5" s="1" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="J5" t="n">
         <v>12</v>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="L5" t="n">
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -725,7 +725,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_DOS_VIERNES</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -735,31 +735,31 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I6" s="1" t="n">
-        <v>46332</v>
+        <v>46311</v>
       </c>
       <c r="J6" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46360</v>
+        <v>46311</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -799,16 +799,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I7" s="1" t="n">
-        <v>46354</v>
+        <v>46319</v>
       </c>
       <c r="J7" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46361</v>
+        <v>46326</v>
       </c>
       <c r="L7" t="n">
         <v>2</v>
@@ -820,77 +820,77 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>400CIG028</t>
+          <t>400CID002</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>400CIG029 -3cred- Proyecto de grado I</t>
+          <t>400CID002 - 4cred- Sistemas de Bases de Datos</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Obligatorio</t>
+          <t>ProcesoDesarrollo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I8" s="1" t="n">
-        <v>46234</v>
+        <v>46333</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46234</v>
+        <v>46340</v>
       </c>
       <c r="L8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>400CIG028</t>
+          <t>400CID002</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>400CIG029 -3cred- Proyecto de grado I</t>
+          <t>400CID002 - 4cred- Sistemas de Bases de Datos</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Obligatorio</t>
+          <t>ProcesoDesarrollo</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_DOS_VIERNES</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -900,358 +900,358 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>46248</v>
+        <v>46332</v>
       </c>
       <c r="J9" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46276</v>
+        <v>46353</v>
       </c>
       <c r="L9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M9" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>400CIG028</t>
+          <t>400CID002</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>400CIG029 -3cred- Proyecto de grado I</t>
+          <t>400CID002 - 4cred- Sistemas de Bases de Datos</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Obligatorio</t>
+          <t>ProcesoDesarrollo</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="I10" s="1" t="n">
-        <v>46290</v>
+        <v>46354</v>
       </c>
       <c r="J10" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46325</v>
+        <v>46354</v>
       </c>
       <c r="L10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>400CIG029</t>
+          <t>400CID002</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>400CIG029 -4cred- Proyecto de grado 2</t>
+          <t>400CID002 - 4cred- Sistemas de Bases de Datos</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SoloMiercoles</t>
+          <t>ProcesoDesarrollo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_MIERCOLES</t>
+          <t>FRANJA_UNO_VIERNES</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>miercoles</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>18:30:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>20:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="I11" s="1" t="n">
-        <v>46239</v>
+        <v>46360</v>
       </c>
       <c r="J11" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46274</v>
+        <v>46360</v>
       </c>
       <c r="L11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>400CIG029</t>
+          <t>400CIG028</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>400CIG029 -4cred- Proyecto de grado 2</t>
+          <t>400CIG029 -3cred- Proyecto de grado I</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SoloMiercoles</t>
+          <t>Obligatorio</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_MIERCOLES</t>
+          <t>FRANJA_UNO_VIERNES</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>miercoles</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>18:30:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>20:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I12" s="1" t="n">
-        <v>46288</v>
+        <v>46234</v>
       </c>
       <c r="J12" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46330</v>
+        <v>46234</v>
       </c>
       <c r="L12" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>10.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>400CIG037</t>
+          <t>400CIG028</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>400CIG037 -3cred -Tópicos Avanzados Ing de Software</t>
+          <t>400CIG029 -3cred- Proyecto de grado I</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TemasAvanzados</t>
+          <t>Obligatorio</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_UNO_VIERNES</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I13" s="1" t="n">
-        <v>46242</v>
+        <v>46248</v>
       </c>
       <c r="J13" t="n">
         <v>7</v>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="L13" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M13" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>400CIG037</t>
+          <t>400CIG028</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>400CIG037 -3cred -Tópicos Avanzados Ing de Software</t>
+          <t>400CIG029 -3cred- Proyecto de grado I</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>TemasAvanzados</t>
+          <t>Obligatorio</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>FRANJA_DOS_SABADO</t>
+          <t>FRANJA_UNO_VIERNES</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>46263</v>
+        <v>46290</v>
       </c>
       <c r="J14" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46263</v>
+        <v>46325</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M14" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>400CIG037</t>
+          <t>400CIG029</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>400CIG037 -3cred -Tópicos Avanzados Ing de Software</t>
+          <t>400CIG029 -4cred- Proyecto de grado 2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>TemasAvanzados</t>
+          <t>SoloMiercoles</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_UNO_MIERCOLES</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>miercoles</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>18:30:00</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>20:00:00</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I15" s="1" t="n">
-        <v>46291</v>
+        <v>46239</v>
       </c>
       <c r="J15" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46305</v>
+        <v>46274</v>
       </c>
       <c r="L15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M15" t="n">
         <v>9</v>
@@ -1260,127 +1260,127 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>400CIG037</t>
+          <t>400CIG029</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>400CIG037 -3cred -Tópicos Avanzados Ing de Software</t>
+          <t>400CIG029 -4cred- Proyecto de grado 2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>TemasAvanzados</t>
+          <t>SoloMiercoles</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_UNO_MIERCOLES</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>miercoles</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>18:30:00</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>20:00:00</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="I16" s="1" t="n">
-        <v>46319</v>
+        <v>46288</v>
       </c>
       <c r="J16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46326</v>
+        <v>46330</v>
       </c>
       <c r="L16" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="M16" t="n">
-        <v>6</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>400CIS002</t>
+          <t>400CIG037</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>400CIS002 - 4cred- Arquitectura de software</t>
+          <t>400CIG037 -3cred -Tópicos Avanzados Ing de Software</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ProcesoDesarrollo</t>
+          <t>TemasAvanzados</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>FRANJA_TRES_VIERNES</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>19:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>21:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I17" s="1" t="n">
-        <v>46234</v>
+        <v>46242</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46234</v>
+        <v>46277</v>
       </c>
       <c r="L17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M17" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>400CIS002</t>
+          <t>400CIG037</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>400CIS002 - 4cred- Arquitectura de software</t>
+          <t>400CIG037 -3cred -Tópicos Avanzados Ing de Software</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ProcesoDesarrollo</t>
+          <t>TemasAvanzados</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1404,132 +1404,132 @@
         </is>
       </c>
       <c r="H18" t="n">
+        <v>5</v>
+      </c>
+      <c r="I18" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="J18" t="n">
+        <v>5</v>
+      </c>
+      <c r="K18" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="L18" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="1" t="n">
-        <v>46235</v>
-      </c>
-      <c r="J18" t="n">
-        <v>4</v>
-      </c>
-      <c r="K18" s="1" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L18" t="n">
-        <v>4</v>
-      </c>
       <c r="M18" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>400CIS002</t>
+          <t>400CIG037</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>400CIS002 - 4cred- Arquitectura de software</t>
+          <t>400CIG037 -3cred -Tópicos Avanzados Ing de Software</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ProcesoDesarrollo</t>
+          <t>TemasAvanzados</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>FRANJA_TRES_VIERNES</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>19:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>21:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I19" s="1" t="n">
-        <v>46262</v>
+        <v>46291</v>
       </c>
       <c r="J19" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46276</v>
+        <v>46305</v>
       </c>
       <c r="L19" t="n">
         <v>3</v>
       </c>
       <c r="M19" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>400CIS002</t>
+          <t>400CIG037</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>400CIS002 - 4cred- Arquitectura de software</t>
+          <t>400CIG037 -3cred -Tópicos Avanzados Ing de Software</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ProcesoDesarrollo</t>
+          <t>TemasAvanzados</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>FRANJA_TRES_VIERNES</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>19:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>21:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I20" s="1" t="n">
-        <v>46290</v>
+        <v>46319</v>
       </c>
       <c r="J20" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46360</v>
+        <v>46326</v>
       </c>
       <c r="L20" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="M20" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -1550,41 +1550,41 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>FRANJA_DOS_SABADO</t>
+          <t>FRANJA_TRES_VIERNES</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>21:00:00</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="I21" s="1" t="n">
-        <v>46361</v>
+        <v>46234</v>
       </c>
       <c r="J21" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46361</v>
+        <v>46234</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -1624,33 +1624,33 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="I22" s="1" t="n">
-        <v>46361</v>
+        <v>46235</v>
       </c>
       <c r="J22" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46361</v>
+        <v>46256</v>
       </c>
       <c r="L22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M22" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>400CIS021</t>
+          <t>400CIS002</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>400CIS021 - 4cred- Ingeniería de Requerimientos</t>
+          <t>400CIS002 - 4cred- Arquitectura de software</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1660,52 +1660,52 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_TRES_VIERNES</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>21:00:00</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I23" s="1" t="n">
-        <v>46235</v>
+        <v>46262</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46235</v>
+        <v>46276</v>
       </c>
       <c r="L23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>400CIS021</t>
+          <t>400CIS002</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>400CIS021 - 4cred- Ingeniería de Requerimientos</t>
+          <t>400CIS002 - 4cred- Arquitectura de software</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_TRES_VIERNES</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1725,42 +1725,42 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>21:00:00</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>46234</v>
+        <v>46290</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46234</v>
+        <v>46360</v>
       </c>
       <c r="L24" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="M24" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>400CIS021</t>
+          <t>400CIS002</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>400CIS021 - 4cred- Ingeniería de Requerimientos</t>
+          <t>400CIS002 - 4cred- Arquitectura de software</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1770,52 +1770,52 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>FRANJA_DOS_VIERNES</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>19:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="I25" s="1" t="n">
-        <v>46248</v>
+        <v>46361</v>
       </c>
       <c r="J25" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46255</v>
+        <v>46361</v>
       </c>
       <c r="L25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>400CIS021</t>
+          <t>400CIS002</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>400CIS021 - 4cred- Ingeniería de Requerimientos</t>
+          <t>400CIS002 - 4cred- Arquitectura de software</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1825,41 +1825,41 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_UNO_SABADO</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>07:00:00</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="H26" t="n">
+        <v>19</v>
+      </c>
+      <c r="I26" s="1" t="n">
+        <v>46361</v>
+      </c>
+      <c r="J26" t="n">
+        <v>19</v>
+      </c>
+      <c r="K26" s="1" t="n">
+        <v>46361</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M26" t="n">
         <v>3</v>
-      </c>
-      <c r="I26" s="1" t="n">
-        <v>46248</v>
-      </c>
-      <c r="J26" t="n">
-        <v>5</v>
-      </c>
-      <c r="K26" s="1" t="n">
-        <v>46262</v>
-      </c>
-      <c r="L26" t="n">
-        <v>3</v>
-      </c>
-      <c r="M26" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="27">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1890,25 +1890,25 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I27" s="1" t="n">
-        <v>46270</v>
+        <v>46235</v>
       </c>
       <c r="J27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46270</v>
+        <v>46235</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_DOS_VIERNES</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1945,25 +1945,25 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I28" s="1" t="n">
-        <v>46276</v>
+        <v>46234</v>
       </c>
       <c r="J28" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46276</v>
+        <v>46234</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_DOS_VIERNES</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2000,25 +2000,25 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I29" s="1" t="n">
-        <v>46290</v>
+        <v>46248</v>
       </c>
       <c r="J29" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46304</v>
+        <v>46262</v>
       </c>
       <c r="L29" t="n">
         <v>3</v>
@@ -2045,41 +2045,41 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_TRES_VIERNES</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>21:00:00</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I30" s="1" t="n">
-        <v>46312</v>
+        <v>46248</v>
       </c>
       <c r="J30" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46312</v>
+        <v>46255</v>
       </c>
       <c r="L30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
@@ -2100,41 +2100,41 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_UNO_SABADO</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>07:00:00</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I31" s="1" t="n">
-        <v>46318</v>
+        <v>46270</v>
       </c>
       <c r="J31" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46325</v>
+        <v>46270</v>
       </c>
       <c r="L31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -2155,41 +2155,41 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_DOS_VIERNES</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="I32" s="1" t="n">
-        <v>46333</v>
+        <v>46276</v>
       </c>
       <c r="J32" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46354</v>
+        <v>46276</v>
       </c>
       <c r="L32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -2210,90 +2210,90 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>FRANJA_DOS_SABADO</t>
+          <t>FRANJA_DOS_VIERNES</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I33" s="1" t="n">
-        <v>46347</v>
+        <v>46290</v>
       </c>
       <c r="J33" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46347</v>
+        <v>46304</v>
       </c>
       <c r="L33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M33" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>400FTA005</t>
+          <t>400CIS021</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>400FTA005 -3cred- Ética e Impactos de la Tecnol</t>
+          <t>400CIS021 - 4cred- Ingeniería de Requerimientos</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Obligatorio</t>
+          <t>ProcesoDesarrollo</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_UNO_SABADO</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>07:00:00</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="I34" s="1" t="n">
-        <v>46234</v>
+        <v>46312</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46234</v>
+        <v>46312</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2305,22 +2305,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>400FTA005</t>
+          <t>400CIS021</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>400FTA005 -3cred- Ética e Impactos de la Tecnol</t>
+          <t>400CIS021 - 4cred- Ingeniería de Requerimientos</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Obligatorio</t>
+          <t>ProcesoDesarrollo</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_DOS_VIERNES</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2330,107 +2330,107 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>19:00:00</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="I35" s="1" t="n">
-        <v>46248</v>
+        <v>46318</v>
       </c>
       <c r="J35" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46276</v>
+        <v>46325</v>
       </c>
       <c r="L35" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M35" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>400FTA005</t>
+          <t>400CIS021</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>400FTA005 -3cred- Ética e Impactos de la Tecnol</t>
+          <t>400CIS021 - 4cred- Ingeniería de Requerimientos</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Obligatorio</t>
+          <t>ProcesoDesarrollo</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_VIERNES</t>
+          <t>FRANJA_UNO_SABADO</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sabado</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>07:00:00</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I36" s="1" t="n">
-        <v>46290</v>
+        <v>46333</v>
       </c>
       <c r="J36" t="n">
         <v>18</v>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46353</v>
+        <v>46354</v>
       </c>
       <c r="L36" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="M36" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>400ITA003</t>
+          <t>400CIS021</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>400ITA003 - 3cred - Arquitectura de Software en la nube</t>
+          <t>400CIS021 - 4cred- Ingeniería de Requerimientos</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>TemasAvanzados</t>
+          <t>ProcesoDesarrollo</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2440,80 +2440,80 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I37" s="1" t="n">
-        <v>46242</v>
+        <v>46347</v>
       </c>
       <c r="J37" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46277</v>
+        <v>46347</v>
       </c>
       <c r="L37" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>400ITA003</t>
+          <t>400FTA005</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>400ITA003 - 3cred - Arquitectura de Software en la nube</t>
+          <t>400FTA005 -3cred- Ética e Impactos de la Tecnol</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>TemasAvanzados</t>
+          <t>Obligatorio</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>FRANJA_DOS_SABADO</t>
+          <t>FRANJA_UNO_VIERNES</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I38" s="1" t="n">
-        <v>46263</v>
+        <v>46234</v>
       </c>
       <c r="J38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46263</v>
+        <v>46234</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -2525,122 +2525,122 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>400ITA003</t>
+          <t>400FTA005</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>400ITA003 - 3cred - Arquitectura de Software en la nube</t>
+          <t>400FTA005 -3cred- Ética e Impactos de la Tecnol</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>TemasAvanzados</t>
+          <t>Obligatorio</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_UNO_VIERNES</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I39" s="1" t="n">
-        <v>46291</v>
+        <v>46248</v>
       </c>
       <c r="J39" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46305</v>
+        <v>46276</v>
       </c>
       <c r="L39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M39" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>400ITA003</t>
+          <t>400FTA005</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>400ITA003 - 3cred - Arquitectura de Software en la nube</t>
+          <t>400FTA005 -3cred- Ética e Impactos de la Tecnol</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>TemasAvanzados</t>
+          <t>Obligatorio</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_UNO_VIERNES</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>sabado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>17:00:00</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="I40" s="1" t="n">
-        <v>46319</v>
+        <v>46290</v>
       </c>
       <c r="J40" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46326</v>
+        <v>46353</v>
       </c>
       <c r="L40" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="M40" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>400ITA005</t>
+          <t>400ITA003</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>400ITA005 - 3cred - El Negocio del sw</t>
+          <t>400ITA003 - 3cred - Arquitectura de Software en la nube</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -2690,12 +2690,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>400ITA005</t>
+          <t>400ITA003</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>400ITA005 - 3cred - El Negocio del sw</t>
+          <t>400ITA003 - 3cred - Arquitectura de Software en la nube</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>FRANJA_DOS_SABADO</t>
+          <t>FRANJA_UNO_SABADO</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2715,12 +2715,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
+          <t>07:00:00</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
           <t>10:00:00</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>13:00:00</t>
         </is>
       </c>
       <c r="H42" t="n">
@@ -2745,12 +2745,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>400ITA005</t>
+          <t>400ITA003</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>400ITA005 - 3cred - El Negocio del sw</t>
+          <t>400ITA003 - 3cred - Arquitectura de Software en la nube</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2770,12 +2770,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -2800,12 +2800,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>400ITA005</t>
+          <t>400ITA003</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>400ITA005 - 3cred - El Negocio del sw</t>
+          <t>400ITA003 - 3cred - Arquitectura de Software en la nube</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>FRANJA_UNO_SABADO</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2825,12 +2825,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>07:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H44" t="n">
@@ -2855,22 +2855,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>400ITA007</t>
+          <t>400ITA005</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>400ITA007 - 4cred- Desarrollo de Software seguro</t>
+          <t>400ITA005 - 3cred - El Negocio del sw</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ProcesoDesarrollo</t>
+          <t>TemasAvanzados</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>FRANJA_CUATRO_SABADO</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2880,12 +2880,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>15:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -2904,28 +2904,28 @@
         <v>6</v>
       </c>
       <c r="M45" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>400ITA007</t>
+          <t>400ITA005</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>400ITA007 - 4cred- Desarrollo de Software seguro</t>
+          <t>400ITA005 - 3cred - El Negocio del sw</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ProcesoDesarrollo</t>
+          <t>TemasAvanzados</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>FRANJA_TRES_SABADO</t>
+          <t>FRANJA_UNO_SABADO</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2935,52 +2935,52 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>13:00:00</t>
+          <t>07:00:00</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>15:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I46" s="1" t="n">
-        <v>46242</v>
+        <v>46263</v>
       </c>
       <c r="J46" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46277</v>
+        <v>46263</v>
       </c>
       <c r="L46" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>400ITA007</t>
+          <t>400ITA005</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>400ITA007 - 4cred- Desarrollo de Software seguro</t>
+          <t>400ITA005 - 3cred - El Negocio del sw</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ProcesoDesarrollo</t>
+          <t>TemasAvanzados</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>FRANJA_CUATRO_SABADO</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2990,12 +2990,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>15:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>17:00:00</t>
+          <t>13:00:00</t>
         </is>
       </c>
       <c r="H47" t="n">
@@ -3005,37 +3005,37 @@
         <v>46291</v>
       </c>
       <c r="J47" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46326</v>
+        <v>46305</v>
       </c>
       <c r="L47" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M47" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>400ITA007</t>
+          <t>400ITA005</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>400ITA007 - 4cred- Desarrollo de Software seguro</t>
+          <t>400ITA005 - 3cred - El Negocio del sw</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ProcesoDesarrollo</t>
+          <t>TemasAvanzados</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>FRANJA_TRES_SABADO</t>
+          <t>FRANJA_DOS_SABADO</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3045,19 +3045,19 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
           <t>13:00:00</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>15:00:00</t>
-        </is>
-      </c>
       <c r="H48" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I48" s="1" t="n">
-        <v>46291</v>
+        <v>46319</v>
       </c>
       <c r="J48" t="n">
         <v>14</v>
@@ -3066,9 +3066,229 @@
         <v>46326</v>
       </c>
       <c r="L48" t="n">
+        <v>2</v>
+      </c>
+      <c r="M48" t="n">
         <v>6</v>
       </c>
-      <c r="M48" t="n">
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>400ITA007</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>400ITA007 - 4cred- Desarrollo de Software seguro</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ProcesoDesarrollo</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>FRANJA_CUATRO_SABADO</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>sabado</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>17:00:00</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>2</v>
+      </c>
+      <c r="I49" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="J49" t="n">
+        <v>7</v>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="L49" t="n">
+        <v>6</v>
+      </c>
+      <c r="M49" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>400ITA007</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>400ITA007 - 4cred- Desarrollo de Software seguro</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ProcesoDesarrollo</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>FRANJA_TRES_SABADO</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>sabado</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>13:00:00</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>2</v>
+      </c>
+      <c r="I50" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="J50" t="n">
+        <v>7</v>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="L50" t="n">
+        <v>6</v>
+      </c>
+      <c r="M50" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>400ITA007</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>400ITA007 - 4cred- Desarrollo de Software seguro</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ProcesoDesarrollo</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>FRANJA_CUATRO_SABADO</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>sabado</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>17:00:00</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I51" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J51" t="n">
+        <v>14</v>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="L51" t="n">
+        <v>6</v>
+      </c>
+      <c r="M51" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>400ITA007</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>400ITA007 - 4cred- Desarrollo de Software seguro</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ProcesoDesarrollo</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>FRANJA_TRES_SABADO</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>sabado</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>13:00:00</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>9</v>
+      </c>
+      <c r="I52" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J52" t="n">
+        <v>14</v>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="L52" t="n">
+        <v>6</v>
+      </c>
+      <c r="M52" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>